<commit_message>
feat(processor): add DOCX and ODT document processors with table token support
- Implement AbstractZipTextProcessor base class for ZIP-based text documents
- Add DocxDocumentProcessor with scalar replacement and table token insertion
- Add OdtDocumentProcessor with scalar replacement and table token insertion
- Replace legacy TABLE/COL DSL expansion with token-only pipeline
- Add table anchor mechanism for inserting dynamic tables at token locations
- Update OdsWorkbookProcessor to use new token-based table insertion
- Remove deprecated block expansion logic from spreadsheet processors
- Add proper documentation for all new processor classes and methods
</commit_message>
<xml_diff>
--- a/Book1.xlsx
+++ b/Book1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/onbozoyan/Downloads/report-generator/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{14289FC5-1CE6-3942-9084-81143237FE1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37090526-6C44-2F41-A24A-9D7D07A13C81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3260" yWindow="2160" windowWidth="28040" windowHeight="17440" xr2:uid="{8EE46694-27A0-8048-B457-EF6458B9856F}"/>
   </bookViews>
@@ -35,22 +35,46 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="1">
-  <si>
-    <t>blank</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+  <si>
+    <t>{{token}}</t>
+  </si>
+  <si>
+    <t>Sales report: {{period}}</t>
+  </si>
+  <si>
+    <t>[[TABLE_START:rows]]</t>
+  </si>
+  <si>
+    <t>{{item.name}}</t>
+  </si>
+  <si>
+    <t>{{item.amount}}</t>
+  </si>
+  <si>
+    <t>[[TABLE_END:rows]]</t>
+  </si>
+  <si>
+    <t>Total: {{total}}</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10.5"/>
+      <color rgb="FFFF806C"/>
+      <name val="Monaco"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="2">
@@ -73,8 +97,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -389,12 +414,36 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{219F9550-F4D0-054E-8000-8E802D1DB356}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" t="s">
         <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A3" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A8" s="1" t="s">
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
refactor(generator): simplify ReportData structure and update test cases
- Remove legacy tables and columns fields from ReportData record
- Update all test cases to use simplified ReportData constructor
- Change template file from xlsx to docx in main application
- Add sample data with Russian placeholders for testing
- Remove legacy DSL marker validation test
- Update file paths and names to reflect new test document format
- Modify table ordering logic to address column insertion issues
- Update output file name from sales-report.xlsx to result.docx
</commit_message>
<xml_diff>
--- a/Book1.xlsx
+++ b/Book1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/onbozoyan/Downloads/report-generator/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37090526-6C44-2F41-A24A-9D7D07A13C81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6321F1B4-30E8-3743-8B67-6EA391F97D2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3260" yWindow="2160" windowWidth="28040" windowHeight="17440" xr2:uid="{8EE46694-27A0-8048-B457-EF6458B9856F}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>{{token}}</t>
   </si>
@@ -56,6 +56,9 @@
   </si>
   <si>
     <t>Total: {{total}}</t>
+  </si>
+  <si>
+    <t>{{TABLE_HERE}}</t>
   </si>
 </sst>
 </file>
@@ -414,10 +417,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{219F9550-F4D0-054E-8000-8E802D1DB356}">
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -425,12 +428,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
@@ -441,7 +444,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F7" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>6</v>
       </c>

</xml_diff>